<commit_message>
subimos principio de octubre
</commit_message>
<xml_diff>
--- a/2026/BRIN 2970/Septiembre/Septiembre-BRIN2970.xlsx
+++ b/2026/BRIN 2970/Septiembre/Septiembre-BRIN2970.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemax\Desktop\rc-consorcio2025\2026\BRIN 2970\Septiembre\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\2026\BRIN 2970\Septiembre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8073600F-EA50-4B55-937E-F0152DC05547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E29218A-FA89-4356-86C5-E2D6113AD715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -22,11 +22,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$E$124</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -1256,7 +1251,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="249">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1562,29 +1557,29 @@
     <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="20" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="15" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="15" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="9" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="23" fillId="9" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="23" fillId="9" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1598,12 +1593,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1616,23 +1605,80 @@
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1640,12 +1686,6 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1655,75 +1695,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="20" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1802,9 +1785,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1842,9 +1825,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1877,26 +1860,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1929,26 +1895,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2123,30 +2072,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M128"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.5546875" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13"/>
-      <c r="B1" s="206" t="s">
+      <c r="B1" s="200" t="s">
         <v>134</v>
       </c>
-      <c r="C1" s="206"/>
-      <c r="D1" s="206"/>
+      <c r="C1" s="200"/>
+      <c r="D1" s="200"/>
       <c r="E1" s="46"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
       <c r="B2" s="47" t="s">
         <v>59</v>
@@ -2155,16 +2104,16 @@
       <c r="D2" s="47"/>
       <c r="E2" s="48"/>
     </row>
-    <row r="3" spans="1:5" ht="70.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="70.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14"/>
-      <c r="B3" s="209" t="s">
+      <c r="B3" s="201" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="209"/>
-      <c r="D3" s="209"/>
-      <c r="E3" s="210"/>
-    </row>
-    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="201"/>
+      <c r="D3" s="201"/>
+      <c r="E3" s="202"/>
+    </row>
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
         <v>0</v>
       </c>
@@ -2175,7 +2124,7 @@
       <c r="D4" s="18"/>
       <c r="E4" s="19"/>
     </row>
-    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>57</v>
       </c>
@@ -2188,7 +2137,7 @@
       </c>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="17" t="s">
         <v>58</v>
       </c>
@@ -2199,62 +2148,62 @@
       </c>
       <c r="E6" s="19"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="212" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="204" t="s">
         <v>140</v>
       </c>
-      <c r="C8" s="212"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="212"/>
-      <c r="C9" s="212"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="212"/>
-      <c r="C10" s="212"/>
-    </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="211" t="s">
+      <c r="C8" s="204"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="204"/>
+      <c r="C9" s="204"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="204"/>
+      <c r="C10" s="204"/>
+    </row>
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="203" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="211"/>
-      <c r="C13" s="211"/>
-      <c r="D13" s="211"/>
-      <c r="E13" s="211"/>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="211"/>
-      <c r="B14" s="211"/>
-      <c r="C14" s="211"/>
-      <c r="D14" s="211"/>
-      <c r="E14" s="211"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="211"/>
-      <c r="B15" s="211"/>
-      <c r="C15" s="211"/>
-      <c r="D15" s="211"/>
-      <c r="E15" s="211"/>
-    </row>
-    <row r="16" spans="1:5" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="211"/>
-      <c r="B16" s="211"/>
-      <c r="C16" s="211"/>
-      <c r="D16" s="211"/>
-      <c r="E16" s="211"/>
-    </row>
-    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="203"/>
+      <c r="C13" s="203"/>
+      <c r="D13" s="203"/>
+      <c r="E13" s="203"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="203"/>
+      <c r="B14" s="203"/>
+      <c r="C14" s="203"/>
+      <c r="D14" s="203"/>
+      <c r="E14" s="203"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="203"/>
+      <c r="B15" s="203"/>
+      <c r="C15" s="203"/>
+      <c r="D15" s="203"/>
+      <c r="E15" s="203"/>
+    </row>
+    <row r="16" spans="1:5" ht="127.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="203"/>
+      <c r="B16" s="203"/>
+      <c r="C16" s="203"/>
+      <c r="D16" s="203"/>
+      <c r="E16" s="203"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D17" s="62"/>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="D18" s="62"/>
     </row>
-    <row r="19" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D19" s="62"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>9</v>
       </c>
@@ -2263,7 +2212,7 @@
       <c r="D20" s="66"/>
       <c r="E20" s="12"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
         <v>25</v>
       </c>
@@ -2272,7 +2221,7 @@
       <c r="D21" s="24"/>
       <c r="E21" s="24"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="52" t="s">
         <v>60</v>
       </c>
@@ -2283,7 +2232,7 @@
       <c r="D22" s="107"/>
       <c r="E22" s="5"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>46</v>
       </c>
@@ -2292,7 +2241,7 @@
       <c r="D23" s="107"/>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>47</v>
       </c>
@@ -2301,7 +2250,7 @@
       <c r="D24" s="107"/>
       <c r="E24" s="5"/>
     </row>
-    <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="42" t="s">
         <v>26</v>
       </c>
@@ -2314,7 +2263,7 @@
       <c r="E25" s="79"/>
       <c r="G25" s="20"/>
     </row>
-    <row r="26" spans="1:7" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>31</v>
       </c>
@@ -2323,28 +2272,28 @@
       <c r="D26" s="107"/>
       <c r="E26" s="5"/>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="21"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="107"/>
       <c r="E27" s="5"/>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="107"/>
       <c r="E28" s="5"/>
     </row>
-    <row r="29" spans="1:7" ht="0.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="0.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="124"/>
       <c r="E29" s="5"/>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="42" t="s">
         <v>26</v>
       </c>
@@ -2356,7 +2305,7 @@
       </c>
       <c r="E30" s="79"/>
     </row>
-    <row r="31" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="22" t="s">
         <v>1</v>
       </c>
@@ -2369,7 +2318,7 @@
       </c>
       <c r="F31" s="20"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="25" t="s">
         <v>17</v>
       </c>
@@ -2378,11 +2327,11 @@
       <c r="D32" s="111"/>
       <c r="E32" s="81"/>
     </row>
-    <row r="33" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="207" t="s">
+    <row r="33" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="193" t="s">
         <v>147</v>
       </c>
-      <c r="B33" s="208"/>
+      <c r="B33" s="194"/>
       <c r="C33" s="39"/>
       <c r="D33" s="107">
         <v>50000</v>
@@ -2391,11 +2340,11 @@
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="207" t="s">
+    <row r="34" spans="1:7" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="193" t="s">
         <v>160</v>
       </c>
-      <c r="B34" s="208"/>
+      <c r="B34" s="194"/>
       <c r="C34" s="39"/>
       <c r="D34" s="125">
         <f>350000*2</f>
@@ -2405,7 +2354,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="22" t="s">
         <v>14</v>
       </c>
@@ -2417,7 +2366,7 @@
         <v>750000</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="25" t="s">
         <v>23</v>
       </c>
@@ -2426,11 +2375,11 @@
       <c r="D36" s="119"/>
       <c r="E36" s="84"/>
     </row>
-    <row r="37" spans="1:7" s="28" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="205" t="s">
+    <row r="37" spans="1:7" s="28" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="199" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="205"/>
+      <c r="B37" s="199"/>
       <c r="C37" s="40"/>
       <c r="D37" s="188">
         <v>46625</v>
@@ -2439,7 +2388,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="141" t="s">
         <v>62</v>
       </c>
@@ -2450,7 +2399,7 @@
       </c>
       <c r="E38" s="146"/>
     </row>
-    <row r="39" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="143" t="s">
         <v>2</v>
       </c>
@@ -2462,7 +2411,7 @@
         <v>46625</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="25" t="s">
         <v>15</v>
       </c>
@@ -2471,7 +2420,7 @@
       <c r="D40" s="120"/>
       <c r="E40" s="113"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>33</v>
       </c>
@@ -2485,7 +2434,7 @@
       </c>
       <c r="G41" s="70"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>142</v>
       </c>
@@ -2500,7 +2449,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="str">
         <f>A42</f>
         <v>Sindicatos mes de AGOSTO</v>
@@ -2517,7 +2466,7 @@
         <v>Debito 14/09</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="str">
         <f>A43</f>
         <v>Sindicatos mes de AGOSTO</v>
@@ -2534,7 +2483,7 @@
         <v>Debito 14/09</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="22" t="s">
         <v>3</v>
       </c>
@@ -2546,7 +2495,7 @@
         <v>720385.55999999982</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="25" t="s">
         <v>16</v>
       </c>
@@ -2555,7 +2504,7 @@
       <c r="D46" s="120"/>
       <c r="E46" s="113"/>
     </row>
-    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="52" t="s">
         <v>65</v>
       </c>
@@ -2568,7 +2517,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="144" t="s">
         <v>67</v>
       </c>
@@ -2581,7 +2530,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="144" t="s">
         <v>64</v>
       </c>
@@ -2594,7 +2543,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="22" t="s">
         <v>4</v>
       </c>
@@ -2606,14 +2555,14 @@
         <v>1080916.6500000001</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="25"/>
       <c r="B51" s="22"/>
       <c r="C51" s="22"/>
       <c r="D51" s="118"/>
       <c r="E51" s="114"/>
     </row>
-    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="139" t="s">
         <v>63</v>
       </c>
@@ -2626,7 +2575,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="139" t="s">
         <v>145</v>
       </c>
@@ -2639,7 +2588,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="139" t="s">
         <v>66</v>
       </c>
@@ -2650,11 +2599,11 @@
       </c>
       <c r="E54" s="104"/>
     </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="203" t="s">
+    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="197" t="s">
         <v>144</v>
       </c>
-      <c r="B55" s="204"/>
+      <c r="B55" s="198"/>
       <c r="C55" s="5"/>
       <c r="D55" s="112">
         <v>1100331.6299999999</v>
@@ -2663,11 +2612,11 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="213" t="s">
+    <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="189" t="s">
         <v>149</v>
       </c>
-      <c r="B56" s="214"/>
+      <c r="B56" s="190"/>
       <c r="C56" s="5"/>
       <c r="D56" s="112">
         <v>305000</v>
@@ -2676,7 +2625,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="139" t="s">
         <v>146</v>
       </c>
@@ -2689,7 +2638,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="22" t="s">
         <v>8</v>
       </c>
@@ -2701,7 +2650,7 @@
         <v>1695931.63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="25" t="s">
         <v>10</v>
       </c>
@@ -2710,7 +2659,7 @@
       <c r="D59" s="110"/>
       <c r="E59" s="86"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>165</v>
       </c>
@@ -2722,7 +2671,7 @@
       </c>
       <c r="E60" s="87"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>39</v>
       </c>
@@ -2733,7 +2682,7 @@
       </c>
       <c r="E61" s="29"/>
     </row>
-    <row r="62" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="38" t="s">
         <v>14</v>
       </c>
@@ -2745,14 +2694,14 @@
         <v>83868.25</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
       <c r="D63" s="52"/>
       <c r="E63" s="59"/>
     </row>
-    <row r="64" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="23" t="s">
         <v>56</v>
       </c>
@@ -2763,13 +2712,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
       <c r="D65" s="62"/>
       <c r="E65" s="63"/>
       <c r="F65" s="31"/>
     </row>
-    <row r="66" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>11</v>
       </c>
@@ -2788,7 +2737,7 @@
       <c r="K66" s="70"/>
       <c r="L66" s="70"/>
     </row>
-    <row r="67" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D67" s="62"/>
       <c r="E67" s="62"/>
       <c r="H67" s="70"/>
@@ -2797,7 +2746,7 @@
       <c r="K67" s="70"/>
       <c r="L67" s="70"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
         <v>129</v>
       </c>
@@ -2811,9 +2760,9 @@
       <c r="K68" s="70"/>
       <c r="L68" s="70"/>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" s="217"/>
-      <c r="B69" s="218"/>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="195"/>
+      <c r="B69" s="196"/>
       <c r="C69" s="5"/>
       <c r="D69" s="112"/>
       <c r="E69" s="104"/>
@@ -2823,9 +2772,9 @@
       <c r="K69" s="70"/>
       <c r="L69" s="70"/>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" s="217"/>
-      <c r="B70" s="218"/>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" s="195"/>
+      <c r="B70" s="196"/>
       <c r="C70" s="5"/>
       <c r="D70" s="112"/>
       <c r="E70" s="54"/>
@@ -2835,7 +2784,7 @@
       <c r="K70" s="70"/>
       <c r="L70" s="70"/>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="55"/>
       <c r="B71" s="57"/>
       <c r="C71" s="5"/>
@@ -2847,7 +2796,7 @@
       <c r="K71" s="70"/>
       <c r="L71" s="70"/>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="36"/>
       <c r="B72" s="35"/>
       <c r="C72" s="35"/>
@@ -2862,7 +2811,7 @@
       <c r="K72" s="70"/>
       <c r="L72" s="70"/>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D73" s="62"/>
       <c r="E73" s="62"/>
       <c r="H73" s="70"/>
@@ -2871,12 +2820,12 @@
       <c r="K73" s="70"/>
       <c r="L73" s="70"/>
     </row>
-    <row r="74" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D74" s="62"/>
       <c r="E74" s="62"/>
       <c r="H74" s="91"/>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="9" t="s">
         <v>32</v>
       </c>
@@ -2885,28 +2834,28 @@
       <c r="D75" s="66"/>
       <c r="E75" s="67"/>
     </row>
-    <row r="76" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="213"/>
-      <c r="B76" s="214"/>
+    <row r="76" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="189"/>
+      <c r="B76" s="190"/>
       <c r="C76" s="5"/>
       <c r="D76" s="112"/>
       <c r="E76" s="104"/>
     </row>
-    <row r="77" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="207"/>
-      <c r="B77" s="208"/>
+    <row r="77" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="193"/>
+      <c r="B77" s="194"/>
       <c r="C77" s="5"/>
       <c r="D77" s="56"/>
       <c r="E77" s="54"/>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" s="55"/>
       <c r="B78" s="57"/>
       <c r="C78" s="5"/>
       <c r="D78" s="56"/>
       <c r="E78" s="54"/>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A79" s="36"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -2916,13 +2865,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D80" s="62"/>
     </row>
-    <row r="81" spans="1:5" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D81" s="62"/>
     </row>
-    <row r="82" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="105" t="s">
         <v>168</v>
       </c>
@@ -2933,10 +2882,10 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D83" s="62"/>
     </row>
-    <row r="84" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
         <v>18</v>
       </c>
@@ -2948,10 +2897,10 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D85" s="62"/>
     </row>
-    <row r="86" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A86" s="50" t="s">
         <v>12</v>
       </c>
@@ -2961,7 +2910,7 @@
       </c>
       <c r="D86" s="62"/>
     </row>
-    <row r="87" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A87" s="50" t="s">
         <v>13</v>
       </c>
@@ -2971,7 +2920,7 @@
       </c>
       <c r="D87" s="62"/>
     </row>
-    <row r="88" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A88" s="50" t="s">
         <v>19</v>
       </c>
@@ -2981,7 +2930,7 @@
       </c>
       <c r="D88" s="62"/>
     </row>
-    <row r="89" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A89" s="50" t="s">
         <v>30</v>
       </c>
@@ -2991,19 +2940,19 @@
       </c>
       <c r="D89" s="62"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D90" s="62"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D91" s="62"/>
     </row>
-    <row r="92" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92"/>
       <c r="B92" s="30"/>
       <c r="C92" s="27"/>
       <c r="D92"/>
     </row>
-    <row r="93" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="71" t="s">
         <v>139</v>
       </c>
@@ -3013,7 +2962,7 @@
       <c r="C93" s="27"/>
       <c r="D93" s="34"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="40" t="s">
         <v>36</v>
       </c>
@@ -3023,7 +2972,7 @@
       </c>
       <c r="E94" s="31"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="40" t="s">
         <v>37</v>
       </c>
@@ -3031,7 +2980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="40" t="s">
         <v>130</v>
       </c>
@@ -3040,7 +2989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" ht="71.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="40" t="s">
         <v>166</v>
       </c>
@@ -3048,7 +2997,7 @@
         <v>1660175</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="40" t="s">
         <v>152</v>
       </c>
@@ -3056,7 +3005,7 @@
         <v>-5000000</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="40" t="s">
         <v>38</v>
       </c>
@@ -3065,7 +3014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="40" t="s">
         <v>125</v>
       </c>
@@ -3074,7 +3023,7 @@
         <v>6791899.8499999996</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="74" t="s">
         <v>34</v>
       </c>
@@ -3085,12 +3034,12 @@
       <c r="D101" s="30"/>
       <c r="E101" s="31"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="73"/>
       <c r="B102" s="73"/>
       <c r="D102" s="31"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" s="71" t="s">
         <v>126</v>
       </c>
@@ -3098,7 +3047,7 @@
         <v>3341459.67</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="40" t="s">
         <v>167</v>
       </c>
@@ -3106,7 +3055,7 @@
         <v>-75000</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="40" t="s">
         <v>158</v>
       </c>
@@ -3114,7 +3063,7 @@
         <v>-1660175</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="40" t="s">
         <v>138</v>
       </c>
@@ -3122,7 +3071,7 @@
         <v>-1660175</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="40" t="s">
         <v>37</v>
       </c>
@@ -3131,7 +3080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" s="40" t="s">
         <v>127</v>
       </c>
@@ -3140,7 +3089,7 @@
         <v>403710.27</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A109" s="74" t="s">
         <v>34</v>
       </c>
@@ -3149,15 +3098,15 @@
         <v>349819.93999999994</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="73"/>
       <c r="B110" s="73"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" s="73"/>
       <c r="B111" s="73"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="71" t="s">
         <v>153</v>
       </c>
@@ -3165,7 +3114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="40" t="s">
         <v>154</v>
       </c>
@@ -3174,7 +3123,7 @@
         <v>5000000</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="40" t="s">
         <v>155</v>
       </c>
@@ -3183,7 +3132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="40" t="s">
         <v>157</v>
       </c>
@@ -3192,7 +3141,7 @@
         <v>23293.700000000186</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="74" t="s">
         <v>156</v>
       </c>
@@ -3201,28 +3150,28 @@
         <v>5023293.7</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" s="73"/>
       <c r="B117" s="73"/>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" s="73"/>
       <c r="B118" s="73"/>
     </row>
-    <row r="119" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A120" s="216" t="s">
+    <row r="119" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A120" s="192" t="s">
         <v>24</v>
       </c>
-      <c r="B120" s="216"/>
-      <c r="C120" s="216"/>
-    </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A121" s="216"/>
-      <c r="B121" s="216"/>
-      <c r="C121" s="216"/>
-    </row>
-    <row r="122" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B120" s="192"/>
+      <c r="C120" s="192"/>
+    </row>
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A121" s="192"/>
+      <c r="B121" s="192"/>
+      <c r="C121" s="192"/>
+    </row>
+    <row r="122" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="68"/>
       <c r="B122" s="26"/>
       <c r="C122" s="26">
@@ -3230,7 +3179,7 @@
       </c>
       <c r="E122" s="78"/>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" s="32" t="s">
         <v>8</v>
       </c>
@@ -3240,46 +3189,39 @@
       </c>
       <c r="C123" s="33"/>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M124" s="7"/>
     </row>
-    <row r="125" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="215"/>
-      <c r="B125" s="215"/>
-      <c r="C125" s="215"/>
-      <c r="D125" s="215"/>
-      <c r="E125" s="215"/>
-    </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A126" s="215"/>
-      <c r="B126" s="215"/>
-      <c r="C126" s="215"/>
-      <c r="D126" s="215"/>
-      <c r="E126" s="215"/>
-    </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A127" s="215"/>
-      <c r="B127" s="215"/>
-      <c r="C127" s="215"/>
-      <c r="D127" s="215"/>
-      <c r="E127" s="215"/>
-    </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A128" s="215"/>
-      <c r="B128" s="215"/>
-      <c r="C128" s="215"/>
-      <c r="D128" s="215"/>
-      <c r="E128" s="215"/>
+    <row r="125" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="191"/>
+      <c r="B125" s="191"/>
+      <c r="C125" s="191"/>
+      <c r="D125" s="191"/>
+      <c r="E125" s="191"/>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A126" s="191"/>
+      <c r="B126" s="191"/>
+      <c r="C126" s="191"/>
+      <c r="D126" s="191"/>
+      <c r="E126" s="191"/>
+    </row>
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A127" s="191"/>
+      <c r="B127" s="191"/>
+      <c r="C127" s="191"/>
+      <c r="D127" s="191"/>
+      <c r="E127" s="191"/>
+    </row>
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A128" s="191"/>
+      <c r="B128" s="191"/>
+      <c r="C128" s="191"/>
+      <c r="D128" s="191"/>
+      <c r="E128" s="191"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A125:E128"/>
-    <mergeCell ref="A120:C121"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A70:B70"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="B1:D1"/>
@@ -3288,6 +3230,13 @@
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="A13:E16"/>
     <mergeCell ref="B8:C10"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A125:E128"/>
+    <mergeCell ref="A120:C121"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A70:B70"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3298,29 +3247,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.28515625" customWidth="1"/>
-    <col min="2" max="4" width="6.5703125" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" customWidth="1"/>
-    <col min="7" max="8" width="8.28515625" customWidth="1"/>
-    <col min="9" max="9" width="8.42578125" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="4.33203125" customWidth="1"/>
+    <col min="2" max="4" width="6.5546875" customWidth="1"/>
+    <col min="5" max="5" width="20.44140625" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" customWidth="1"/>
+    <col min="7" max="8" width="8.33203125" customWidth="1"/>
+    <col min="9" max="9" width="8.44140625" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" customWidth="1"/>
+    <col min="11" max="11" width="13.44140625" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
-    <col min="15" max="15" width="11.28515625" customWidth="1"/>
-    <col min="16" max="18" width="12.42578125" customWidth="1"/>
-    <col min="19" max="19" width="14.7109375" customWidth="1"/>
-    <col min="20" max="20" width="14.28515625" customWidth="1"/>
-    <col min="21" max="21" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.109375" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" customWidth="1"/>
+    <col min="16" max="18" width="12.44140625" customWidth="1"/>
+    <col min="19" max="19" width="14.6640625" customWidth="1"/>
+    <col min="20" max="20" width="14.33203125" customWidth="1"/>
+    <col min="21" max="21" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -3328,21 +3277,21 @@
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
-      <c r="H1" s="238"/>
-      <c r="I1" s="238"/>
-      <c r="J1" s="238"/>
-      <c r="K1" s="238"/>
-      <c r="L1" s="238"/>
-      <c r="M1" s="238"/>
-      <c r="N1" s="238"/>
-      <c r="O1" s="238"/>
-      <c r="P1" s="238"/>
-      <c r="Q1" s="238"/>
-      <c r="R1" s="238"/>
-      <c r="S1" s="238"/>
+      <c r="H1" s="205"/>
+      <c r="I1" s="205"/>
+      <c r="J1" s="205"/>
+      <c r="K1" s="205"/>
+      <c r="L1" s="205"/>
+      <c r="M1" s="205"/>
+      <c r="N1" s="205"/>
+      <c r="O1" s="205"/>
+      <c r="P1" s="205"/>
+      <c r="Q1" s="205"/>
+      <c r="R1" s="205"/>
+      <c r="S1" s="205"/>
       <c r="T1" s="6"/>
     </row>
-    <row r="2" spans="1:23" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -3350,38 +3299,38 @@
       <c r="E2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="237">
+      <c r="F2" s="220">
         <v>1500000</v>
       </c>
-      <c r="G2" s="237"/>
+      <c r="G2" s="220"/>
       <c r="H2" s="168"/>
       <c r="I2" s="168"/>
       <c r="J2" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="226">
-        <v>0</v>
-      </c>
-      <c r="L2" s="226"/>
-      <c r="M2" s="226"/>
+      <c r="K2" s="221">
+        <v>0</v>
+      </c>
+      <c r="L2" s="221"/>
+      <c r="M2" s="221"/>
       <c r="N2" s="15"/>
       <c r="O2" s="15"/>
       <c r="P2" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="Q2" s="237">
+      <c r="Q2" s="220">
         <f>V2</f>
         <v>4377727.09</v>
       </c>
-      <c r="R2" s="237"/>
-      <c r="S2" s="237"/>
+      <c r="R2" s="220"/>
+      <c r="S2" s="220"/>
       <c r="T2" s="41"/>
       <c r="U2" s="20"/>
       <c r="V2">
         <v>4377727.09</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="13.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -3406,186 +3355,186 @@
         <v>3320350</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="241" t="s">
+    <row r="4" spans="1:23" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="212" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="242"/>
-      <c r="C4" s="242"/>
-      <c r="D4" s="242"/>
-      <c r="E4" s="242"/>
-      <c r="F4" s="242"/>
-      <c r="G4" s="242"/>
-      <c r="H4" s="242"/>
-      <c r="I4" s="242"/>
-      <c r="J4" s="242"/>
-      <c r="K4" s="242"/>
-      <c r="L4" s="242"/>
-      <c r="M4" s="242"/>
-      <c r="N4" s="242"/>
-      <c r="O4" s="242"/>
-      <c r="P4" s="242"/>
-      <c r="Q4" s="242"/>
-      <c r="R4" s="242"/>
-      <c r="S4" s="242"/>
-      <c r="T4" s="243"/>
-    </row>
-    <row r="5" spans="1:23" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="244"/>
-      <c r="B5" s="245"/>
-      <c r="C5" s="245"/>
-      <c r="D5" s="245"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="245"/>
-      <c r="G5" s="245"/>
-      <c r="H5" s="245"/>
-      <c r="I5" s="245"/>
-      <c r="J5" s="245"/>
-      <c r="K5" s="245"/>
-      <c r="L5" s="245"/>
-      <c r="M5" s="245"/>
-      <c r="N5" s="245"/>
-      <c r="O5" s="245"/>
-      <c r="P5" s="245"/>
-      <c r="Q5" s="245"/>
-      <c r="R5" s="245"/>
-      <c r="S5" s="245"/>
-      <c r="T5" s="246"/>
-    </row>
-    <row r="6" spans="1:23" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="244"/>
-      <c r="B6" s="245"/>
-      <c r="C6" s="245"/>
-      <c r="D6" s="245"/>
-      <c r="E6" s="245"/>
-      <c r="F6" s="245"/>
-      <c r="G6" s="245"/>
-      <c r="H6" s="245"/>
-      <c r="I6" s="245"/>
-      <c r="J6" s="245"/>
-      <c r="K6" s="245"/>
-      <c r="L6" s="245"/>
-      <c r="M6" s="245"/>
-      <c r="N6" s="245"/>
-      <c r="O6" s="245"/>
-      <c r="P6" s="245"/>
-      <c r="Q6" s="245"/>
-      <c r="R6" s="245"/>
-      <c r="S6" s="245"/>
-      <c r="T6" s="246"/>
-    </row>
-    <row r="7" spans="1:23" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="244"/>
-      <c r="B7" s="245"/>
-      <c r="C7" s="245"/>
-      <c r="D7" s="245"/>
-      <c r="E7" s="245"/>
-      <c r="F7" s="245"/>
-      <c r="G7" s="245"/>
-      <c r="H7" s="245"/>
-      <c r="I7" s="245"/>
-      <c r="J7" s="245"/>
-      <c r="K7" s="245"/>
-      <c r="L7" s="245"/>
-      <c r="M7" s="245"/>
-      <c r="N7" s="245"/>
-      <c r="O7" s="245"/>
-      <c r="P7" s="245"/>
-      <c r="Q7" s="245"/>
-      <c r="R7" s="245"/>
-      <c r="S7" s="245"/>
-      <c r="T7" s="246"/>
-    </row>
-    <row r="8" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="230" t="s">
+      <c r="B4" s="213"/>
+      <c r="C4" s="213"/>
+      <c r="D4" s="213"/>
+      <c r="E4" s="213"/>
+      <c r="F4" s="213"/>
+      <c r="G4" s="213"/>
+      <c r="H4" s="213"/>
+      <c r="I4" s="213"/>
+      <c r="J4" s="213"/>
+      <c r="K4" s="213"/>
+      <c r="L4" s="213"/>
+      <c r="M4" s="213"/>
+      <c r="N4" s="213"/>
+      <c r="O4" s="213"/>
+      <c r="P4" s="213"/>
+      <c r="Q4" s="213"/>
+      <c r="R4" s="213"/>
+      <c r="S4" s="213"/>
+      <c r="T4" s="214"/>
+    </row>
+    <row r="5" spans="1:23" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="215"/>
+      <c r="B5" s="216"/>
+      <c r="C5" s="216"/>
+      <c r="D5" s="216"/>
+      <c r="E5" s="216"/>
+      <c r="F5" s="216"/>
+      <c r="G5" s="216"/>
+      <c r="H5" s="216"/>
+      <c r="I5" s="216"/>
+      <c r="J5" s="216"/>
+      <c r="K5" s="216"/>
+      <c r="L5" s="216"/>
+      <c r="M5" s="216"/>
+      <c r="N5" s="216"/>
+      <c r="O5" s="216"/>
+      <c r="P5" s="216"/>
+      <c r="Q5" s="216"/>
+      <c r="R5" s="216"/>
+      <c r="S5" s="216"/>
+      <c r="T5" s="217"/>
+    </row>
+    <row r="6" spans="1:23" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="215"/>
+      <c r="B6" s="216"/>
+      <c r="C6" s="216"/>
+      <c r="D6" s="216"/>
+      <c r="E6" s="216"/>
+      <c r="F6" s="216"/>
+      <c r="G6" s="216"/>
+      <c r="H6" s="216"/>
+      <c r="I6" s="216"/>
+      <c r="J6" s="216"/>
+      <c r="K6" s="216"/>
+      <c r="L6" s="216"/>
+      <c r="M6" s="216"/>
+      <c r="N6" s="216"/>
+      <c r="O6" s="216"/>
+      <c r="P6" s="216"/>
+      <c r="Q6" s="216"/>
+      <c r="R6" s="216"/>
+      <c r="S6" s="216"/>
+      <c r="T6" s="217"/>
+    </row>
+    <row r="7" spans="1:23" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="215"/>
+      <c r="B7" s="216"/>
+      <c r="C7" s="216"/>
+      <c r="D7" s="216"/>
+      <c r="E7" s="216"/>
+      <c r="F7" s="216"/>
+      <c r="G7" s="216"/>
+      <c r="H7" s="216"/>
+      <c r="I7" s="216"/>
+      <c r="J7" s="216"/>
+      <c r="K7" s="216"/>
+      <c r="L7" s="216"/>
+      <c r="M7" s="216"/>
+      <c r="N7" s="216"/>
+      <c r="O7" s="216"/>
+      <c r="P7" s="216"/>
+      <c r="Q7" s="216"/>
+      <c r="R7" s="216"/>
+      <c r="S7" s="216"/>
+      <c r="T7" s="217"/>
+    </row>
+    <row r="8" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="206" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="221" t="s">
+      <c r="B8" s="208" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="221" t="s">
+      <c r="C8" s="208" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="221" t="s">
+      <c r="D8" s="208" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="221" t="s">
+      <c r="E8" s="208" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="221" t="s">
+      <c r="F8" s="208" t="s">
         <v>112</v>
       </c>
-      <c r="G8" s="221" t="s">
+      <c r="G8" s="208" t="s">
         <v>113</v>
       </c>
-      <c r="H8" s="230" t="s">
+      <c r="H8" s="206" t="s">
         <v>111</v>
       </c>
       <c r="I8" s="148" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="230" t="s">
+      <c r="J8" s="206" t="s">
         <v>35</v>
       </c>
-      <c r="K8" s="221" t="s">
+      <c r="K8" s="208" t="s">
         <v>7</v>
       </c>
-      <c r="L8" s="221" t="s">
+      <c r="L8" s="208" t="s">
         <v>122</v>
       </c>
-      <c r="M8" s="239" t="s">
+      <c r="M8" s="210" t="s">
         <v>22</v>
       </c>
-      <c r="N8" s="230" t="s">
+      <c r="N8" s="206" t="s">
         <v>133</v>
       </c>
-      <c r="O8" s="230" t="s">
+      <c r="O8" s="206" t="s">
         <v>55</v>
       </c>
-      <c r="P8" s="230" t="s">
+      <c r="P8" s="206" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="230" t="s">
+      <c r="Q8" s="206" t="s">
         <v>42</v>
       </c>
-      <c r="R8" s="219" t="s">
+      <c r="R8" s="230" t="s">
         <v>132</v>
       </c>
       <c r="S8" s="149" t="s">
         <v>28</v>
       </c>
-      <c r="T8" s="247" t="s">
+      <c r="T8" s="218" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="231"/>
-      <c r="B9" s="222"/>
-      <c r="C9" s="222"/>
-      <c r="D9" s="222"/>
-      <c r="E9" s="222"/>
-      <c r="F9" s="222"/>
-      <c r="G9" s="222"/>
-      <c r="H9" s="231"/>
+    <row r="9" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="207"/>
+      <c r="B9" s="209"/>
+      <c r="C9" s="209"/>
+      <c r="D9" s="209"/>
+      <c r="E9" s="209"/>
+      <c r="F9" s="209"/>
+      <c r="G9" s="209"/>
+      <c r="H9" s="207"/>
       <c r="I9" s="161" t="s">
         <v>110</v>
       </c>
-      <c r="J9" s="231"/>
-      <c r="K9" s="222"/>
-      <c r="L9" s="222"/>
-      <c r="M9" s="240"/>
-      <c r="N9" s="231"/>
-      <c r="O9" s="231"/>
-      <c r="P9" s="231"/>
-      <c r="Q9" s="231"/>
-      <c r="R9" s="220"/>
+      <c r="J9" s="207"/>
+      <c r="K9" s="209"/>
+      <c r="L9" s="209"/>
+      <c r="M9" s="211"/>
+      <c r="N9" s="207"/>
+      <c r="O9" s="207"/>
+      <c r="P9" s="207"/>
+      <c r="Q9" s="207"/>
+      <c r="R9" s="231"/>
       <c r="S9" s="186" t="str">
         <f>RESUMEN!B8</f>
         <v>VTO 16/10</v>
       </c>
-      <c r="T9" s="248"/>
-    </row>
-    <row r="10" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T9" s="219"/>
+    </row>
+    <row r="10" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="166">
         <v>19</v>
       </c>
@@ -3657,60 +3606,60 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="202">
+    <row r="11" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="155">
         <v>20</v>
       </c>
-      <c r="B11" s="189"/>
-      <c r="C11" s="189"/>
-      <c r="D11" s="189" t="s">
+      <c r="B11" s="131"/>
+      <c r="C11" s="131"/>
+      <c r="D11" s="131" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="190" t="s">
+      <c r="E11" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="F11" s="191">
+      <c r="F11" s="132">
         <v>2.87</v>
       </c>
-      <c r="G11" s="191"/>
-      <c r="H11" s="192"/>
-      <c r="I11" s="193">
+      <c r="G11" s="132"/>
+      <c r="H11" s="235"/>
+      <c r="I11" s="236">
         <f t="shared" ref="I11:I33" si="4">SUM(F11:H11)</f>
         <v>2.87</v>
       </c>
-      <c r="J11" s="194">
+      <c r="J11" s="99">
         <v>173340.2</v>
       </c>
-      <c r="K11" s="194">
+      <c r="K11" s="99">
         <f t="shared" si="0"/>
         <v>173340.2</v>
       </c>
-      <c r="L11" s="195" t="s">
+      <c r="L11" s="117" t="s">
         <v>123</v>
       </c>
-      <c r="M11" s="196">
+      <c r="M11" s="237">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N11" s="197">
+      <c r="N11" s="238">
         <f t="shared" ref="N11:N33" si="5">IF(M11&gt;0,M11*2%,0)</f>
         <v>0</v>
       </c>
-      <c r="O11" s="196"/>
-      <c r="P11" s="198">
+      <c r="O11" s="237"/>
+      <c r="P11" s="239">
         <f t="shared" ref="P11:P33" si="6">Q$2*I11/100</f>
         <v>125640.76748299999</v>
       </c>
-      <c r="Q11" s="199">
+      <c r="Q11" s="240">
         <f t="shared" ref="Q11:Q33" si="7">F$2*I11/100</f>
         <v>43050</v>
       </c>
-      <c r="R11" s="199"/>
-      <c r="S11" s="200">
+      <c r="R11" s="240"/>
+      <c r="S11" s="241">
         <f t="shared" ref="S11:S26" si="8">ROUND(SUM(M11:R11),0) + U11</f>
         <v>168691.20000000001</v>
       </c>
-      <c r="T11" s="201">
+      <c r="T11" s="242">
         <f t="shared" si="2"/>
         <v>173752.2</v>
       </c>
@@ -3722,7 +3671,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="155">
         <v>21</v>
       </c>
@@ -3794,7 +3743,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="154">
         <v>22</v>
       </c>
@@ -3860,7 +3809,7 @@
       </c>
       <c r="W13" s="31"/>
     </row>
-    <row r="14" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="154">
         <v>23</v>
       </c>
@@ -3934,7 +3883,7 @@
       </c>
       <c r="W14" s="31"/>
     </row>
-    <row r="15" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="154">
         <v>24</v>
       </c>
@@ -3999,7 +3948,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="154" t="s">
         <v>68</v>
       </c>
@@ -4065,7 +4014,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="154">
         <v>25</v>
       </c>
@@ -4137,7 +4086,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="154">
         <f>A17+1</f>
         <v>26</v>
@@ -4210,7 +4159,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="154">
         <f t="shared" ref="A19:A27" si="12">A18+1</f>
         <v>27</v>
@@ -4279,7 +4228,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="154">
         <f t="shared" si="12"/>
         <v>28</v>
@@ -4352,7 +4301,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="154">
         <f t="shared" si="12"/>
         <v>29</v>
@@ -4425,7 +4374,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="154">
         <f t="shared" si="12"/>
         <v>30</v>
@@ -4491,7 +4440,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="154">
         <f t="shared" si="12"/>
         <v>31</v>
@@ -4564,7 +4513,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="154">
         <f t="shared" si="12"/>
         <v>32</v>
@@ -4630,7 +4579,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="154">
         <f t="shared" si="12"/>
         <v>33</v>
@@ -4700,7 +4649,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="154">
         <f t="shared" si="12"/>
         <v>34</v>
@@ -4765,7 +4714,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="154">
         <f t="shared" si="12"/>
         <v>35</v>
@@ -4776,10 +4725,10 @@
       <c r="C27" s="130" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="232">
+      <c r="D27" s="225">
         <v>9</v>
       </c>
-      <c r="E27" s="232" t="s">
+      <c r="E27" s="225" t="s">
         <v>107</v>
       </c>
       <c r="F27" s="135">
@@ -4840,7 +4789,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="154" t="s">
         <v>68</v>
       </c>
@@ -4848,8 +4797,8 @@
         <v>5</v>
       </c>
       <c r="C28" s="133"/>
-      <c r="D28" s="233"/>
-      <c r="E28" s="233"/>
+      <c r="D28" s="226"/>
+      <c r="E28" s="226"/>
       <c r="F28" s="135">
         <f>7.73/2</f>
         <v>3.8650000000000002</v>
@@ -4902,7 +4851,7 @@
       </c>
       <c r="U28" s="31"/>
     </row>
-    <row r="29" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="154">
         <v>36</v>
       </c>
@@ -4912,10 +4861,10 @@
       <c r="C29" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="232">
+      <c r="D29" s="225">
         <v>10</v>
       </c>
-      <c r="E29" s="235" t="s">
+      <c r="E29" s="228" t="s">
         <v>108</v>
       </c>
       <c r="F29" s="135">
@@ -4976,7 +4925,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="154" t="s">
         <v>68</v>
       </c>
@@ -4984,8 +4933,8 @@
         <v>18</v>
       </c>
       <c r="C30" s="133"/>
-      <c r="D30" s="233"/>
-      <c r="E30" s="236"/>
+      <c r="D30" s="226"/>
+      <c r="E30" s="229"/>
       <c r="F30" s="135">
         <f>7.73/2</f>
         <v>3.8650000000000002</v>
@@ -5038,7 +4987,7 @@
       </c>
       <c r="U30" s="31"/>
     </row>
-    <row r="31" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="154">
         <v>37</v>
       </c>
@@ -5048,10 +4997,10 @@
       <c r="C31" s="133" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="232" t="s">
+      <c r="D31" s="225" t="s">
         <v>92</v>
       </c>
-      <c r="E31" s="232" t="s">
+      <c r="E31" s="225" t="s">
         <v>109</v>
       </c>
       <c r="F31" s="135">
@@ -5111,7 +5060,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="154" t="s">
         <v>68</v>
       </c>
@@ -5119,8 +5068,8 @@
         <v>3</v>
       </c>
       <c r="C32" s="134"/>
-      <c r="D32" s="234"/>
-      <c r="E32" s="234"/>
+      <c r="D32" s="227"/>
+      <c r="E32" s="227"/>
       <c r="F32" s="135">
         <f>12.13/3</f>
         <v>4.0433333333333339</v>
@@ -5168,7 +5117,7 @@
       </c>
       <c r="U32" s="31"/>
     </row>
-    <row r="33" spans="1:21" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" ht="14.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="170" t="s">
         <v>68</v>
       </c>
@@ -5176,8 +5125,8 @@
         <v>16</v>
       </c>
       <c r="C33" s="134"/>
-      <c r="D33" s="234"/>
-      <c r="E33" s="234"/>
+      <c r="D33" s="227"/>
+      <c r="E33" s="227"/>
       <c r="F33" s="135">
         <f>12.13/3</f>
         <v>4.0433333333333339</v>
@@ -5225,14 +5174,14 @@
       </c>
       <c r="U33" s="31"/>
     </row>
-    <row r="34" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="227" t="s">
+    <row r="34" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="228"/>
-      <c r="C34" s="228"/>
-      <c r="D34" s="228"/>
-      <c r="E34" s="229"/>
+      <c r="B34" s="223"/>
+      <c r="C34" s="223"/>
+      <c r="D34" s="223"/>
+      <c r="E34" s="224"/>
       <c r="F34" s="179"/>
       <c r="G34" s="179"/>
       <c r="H34" s="180">
@@ -5282,7 +5231,7 @@
         <v>6060669.5599999996</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E35" s="37"/>
       <c r="F35" s="37"/>
       <c r="G35" s="37"/>
@@ -5294,14 +5243,14 @@
         <v>6791899.8499999996</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A36" s="223"/>
-      <c r="B36" s="223"/>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A36" s="232"/>
+      <c r="B36" s="232"/>
       <c r="C36" s="128"/>
       <c r="D36" s="128"/>
-      <c r="H36" s="224"/>
+      <c r="H36" s="233"/>
       <c r="I36" s="129"/>
-      <c r="J36" s="225"/>
+      <c r="J36" s="234"/>
       <c r="K36" s="102" t="s">
         <v>114</v>
       </c>
@@ -5310,34 +5259,34 @@
         <v>403710.27</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A37" s="223"/>
-      <c r="B37" s="223"/>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A37" s="232"/>
+      <c r="B37" s="232"/>
       <c r="C37" s="128"/>
       <c r="D37" s="128"/>
-      <c r="H37" s="224"/>
+      <c r="H37" s="233"/>
       <c r="I37" s="129"/>
-      <c r="J37" s="225"/>
+      <c r="J37" s="234"/>
       <c r="K37" s="103"/>
       <c r="L37" s="103"/>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="J48">
         <f>SUM(H46:H47)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J52">
         <f>SUM(H50:H51)</f>
         <v>0</v>
@@ -5345,6 +5294,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A36:B37"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="H1:S1"/>
     <mergeCell ref="N8:N9"/>
     <mergeCell ref="J8:J9"/>
@@ -5361,23 +5327,6 @@
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
     <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="A36:B37"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="J36:J37"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5388,9 +5337,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D7123E2-E76E-40B2-9631-974509386176}">
   <dimension ref="C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="3" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>136</v>
       </c>

</xml_diff>